<commit_message>
Detection of runtime - python or pyscript. Move the get rates from NBP operation to async and depending on runtime.
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -7,7 +7,8 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Dividend Tax" sheetId="1" r:id="rId1"/>
+    <sheet name="Sale Tax" sheetId="1" r:id="rId1"/>
+    <sheet name="Dividend Tax" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,6 +20,107 @@
     <author/>
   </authors>
   <commentList>
+    <comment ref="L1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>= Shares * PurchasePrice USD * PurchaseUSDRate D-1 PLN</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>= FeesAndCommissions USD * SaleUSDRate D-1 PLN</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>= GrossProceeds USD * SaleUSDRate D-1 PLN</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>= sum(PurchaseCost PLN) + sum(FeesAndCommissions PLN)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>= ( sum(GrossProceeds PLN) - TotalCost PL ) * 0,19</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Into Pit38 C.22</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="8"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Into Pit38 C.23</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
     <comment ref="E1" authorId="0">
       <text>
         <r>
@@ -71,7 +173,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F4" authorId="0">
+    <comment ref="F3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -84,7 +186,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G4" authorId="0">
+    <comment ref="G3" authorId="0">
       <text>
         <r>
           <rPr>
@@ -102,7 +204,64 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="27">
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t>PurchaseDate</t>
+  </si>
+  <si>
+    <t>PurchasePrice USD</t>
+  </si>
+  <si>
+    <t>PurchaseUSDRate D-1 PLN</t>
+  </si>
+  <si>
+    <t>SaleDate</t>
+  </si>
+  <si>
+    <t>SalePrice USD</t>
+  </si>
+  <si>
+    <t>GrossProceeds USD</t>
+  </si>
+  <si>
+    <t>Amount USD</t>
+  </si>
+  <si>
+    <t>FeesAndCommissions USD</t>
+  </si>
+  <si>
+    <t>SaleUSDRate D-1 PLN</t>
+  </si>
+  <si>
+    <t>PurchaseCost PLN</t>
+  </si>
+  <si>
+    <t>FeesAndCommissions PLN</t>
+  </si>
+  <si>
+    <t>GrossProceeds PLN</t>
+  </si>
+  <si>
+    <t>TotalCost PLN</t>
+  </si>
+  <si>
+    <t>Tax PLN</t>
+  </si>
+  <si>
+    <t>ESPP</t>
+  </si>
+  <si>
+    <t>Div Reinv</t>
+  </si>
+  <si>
+    <t>Sale</t>
+  </si>
   <si>
     <t>DividendDate</t>
   </si>
@@ -165,7 +324,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -181,6 +340,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0FFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF87CEFA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -218,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -226,6 +391,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,7 +687,320 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:P7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" s="2" customFormat="1">
+      <c r="A2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0.8082</v>
+      </c>
+      <c r="C2" s="3">
+        <v>44742</v>
+      </c>
+      <c r="D2" s="2">
+        <v>36.244</v>
+      </c>
+      <c r="E2" s="2">
+        <v>4.4533</v>
+      </c>
+      <c r="F2" s="3">
+        <v>45216</v>
+      </c>
+      <c r="G2" s="2">
+        <v>53.4208</v>
+      </c>
+      <c r="H2" s="2">
+        <v>43.17</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>4.2505</v>
+      </c>
+      <c r="L2" s="2">
+        <v>130.45</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2">
+        <v>183.51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="2" customFormat="1">
+      <c r="A3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="2">
+        <v>7.1697</v>
+      </c>
+      <c r="C3" s="3">
+        <v>44742</v>
+      </c>
+      <c r="D3" s="2">
+        <v>36.244</v>
+      </c>
+      <c r="E3" s="2">
+        <v>4.4533</v>
+      </c>
+      <c r="F3" s="3">
+        <v>45216</v>
+      </c>
+      <c r="G3" s="2">
+        <v>53.4208</v>
+      </c>
+      <c r="H3" s="2">
+        <v>383.01</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>4.2505</v>
+      </c>
+      <c r="L3" s="2">
+        <v>1157.23</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>1627.99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="2" customFormat="1">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3.733</v>
+      </c>
+      <c r="C4" s="3">
+        <v>44862</v>
+      </c>
+      <c r="D4" s="2">
+        <v>44.9465</v>
+      </c>
+      <c r="E4" s="2">
+        <v>4.7216</v>
+      </c>
+      <c r="F4" s="3">
+        <v>45216</v>
+      </c>
+      <c r="G4" s="2">
+        <v>53.4208</v>
+      </c>
+      <c r="H4" s="2">
+        <v>199.42</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>4.2505</v>
+      </c>
+      <c r="L4" s="2">
+        <v>792.21</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0</v>
+      </c>
+      <c r="N4" s="2">
+        <v>847.63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="2" customFormat="1">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2">
+        <v>570.8443</v>
+      </c>
+      <c r="C5" s="3">
+        <v>44925</v>
+      </c>
+      <c r="D5" s="2">
+        <v>36.21</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4.4078</v>
+      </c>
+      <c r="F5" s="3">
+        <v>45216</v>
+      </c>
+      <c r="G5" s="2">
+        <v>53.4208</v>
+      </c>
+      <c r="H5" s="2">
+        <v>30494.96</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2">
+        <v>4.2505</v>
+      </c>
+      <c r="L5" s="2">
+        <v>91110.42999999999</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0</v>
+      </c>
+      <c r="N5" s="2">
+        <v>129618.82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" s="4" customFormat="1">
+      <c r="A6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="4">
+        <v>582.5552</v>
+      </c>
+      <c r="D6" s="4">
+        <v>0</v>
+      </c>
+      <c r="E6" s="4">
+        <v>0</v>
+      </c>
+      <c r="F6" s="5">
+        <v>45216</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4">
+        <v>0</v>
+      </c>
+      <c r="I6" s="4">
+        <v>31120.56</v>
+      </c>
+      <c r="J6" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="K6" s="4">
+        <v>4.2505</v>
+      </c>
+      <c r="L6" s="4">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4">
+        <v>0.21</v>
+      </c>
+      <c r="N6" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" s="6" customFormat="1">
+      <c r="L7" s="6">
+        <v>93190.32000000001</v>
+      </c>
+      <c r="M7" s="6">
+        <v>0.21</v>
+      </c>
+      <c r="N7" s="6">
+        <v>132277.96</v>
+      </c>
+      <c r="O7" s="6">
+        <v>93190.53</v>
+      </c>
+      <c r="P7" s="6">
+        <v>7426.61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -535,88 +1015,65 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="2" customFormat="1">
       <c r="A2" s="3">
-        <v>45042</v>
+        <v>45224</v>
       </c>
       <c r="B2" s="2">
-        <v>152.51</v>
+        <v>418</v>
       </c>
       <c r="C2" s="2">
-        <v>8.130000000000001</v>
+        <v>62.7</v>
       </c>
       <c r="D2" s="2">
-        <v>4.1649</v>
+        <v>4.1884</v>
       </c>
       <c r="E2" s="2">
-        <v>635.1900000000001</v>
+        <v>1750.75</v>
       </c>
       <c r="F2" s="2">
-        <v>33.86</v>
+        <v>262.61</v>
       </c>
       <c r="G2" s="2">
-        <v>120.69</v>
+        <v>332.64</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="2" customFormat="1">
-      <c r="A3" s="3">
-        <v>44951</v>
-      </c>
-      <c r="B3" s="2">
-        <v>5.21</v>
-      </c>
-      <c r="C3" s="2">
-        <v>1.3</v>
-      </c>
-      <c r="D3" s="2">
-        <v>4.3341</v>
-      </c>
-      <c r="E3" s="2">
-        <v>22.58</v>
-      </c>
-      <c r="F3" s="2">
-        <v>5.63</v>
-      </c>
-      <c r="G3" s="2">
-        <v>4.29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="4" customFormat="1">
-      <c r="E4" s="4">
-        <v>657.77</v>
-      </c>
-      <c r="F4" s="4">
-        <v>39.49</v>
-      </c>
-      <c r="G4" s="4">
-        <v>124.98</v>
-      </c>
-      <c r="H4" s="4">
-        <v>85.48</v>
+    <row r="3" spans="1:8" s="6" customFormat="1">
+      <c r="E3" s="6">
+        <v>1750.75</v>
+      </c>
+      <c r="F3" s="6">
+        <v>262.61</v>
+      </c>
+      <c r="G3" s="6">
+        <v>332.64</v>
+      </c>
+      <c r="H3" s="6">
+        <v>70.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>